<commit_message>
Add proxy configuration support for DeepSeek API requests
</commit_message>
<xml_diff>
--- a/TEST2.xlsx
+++ b/TEST2.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="768" yWindow="768" windowWidth="17280" windowHeight="9960" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1950" yWindow="1950" windowWidth="28800" windowHeight="15345" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1 (2)" sheetId="1" state="visible" r:id="rId1"/>
@@ -12,7 +12,7 @@
     <sheet name="Sheet3" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="152511" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -105,7 +105,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment vertical="center"/>
@@ -114,9 +114,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
@@ -527,13 +524,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="15.6"/>
+  <dimension ref="A1:H10"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col width="9" customWidth="1" style="2" min="1" max="3"/>
     <col width="9" bestFit="1" customWidth="1" style="2" min="4" max="4"/>
     <col width="9" customWidth="1" style="2" min="5" max="13"/>
-    <col width="9" customWidth="1" style="6" min="14" max="16384"/>
+    <col width="9" customWidth="1" style="5" min="14" max="14"/>
+    <col width="9" customWidth="1" style="5" min="15" max="16384"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -564,43 +562,53 @@
           <t>系列3</t>
         </is>
       </c>
-      <c r="E2" s="5">
+      <c r="E2" s="4">
         <f>MIN(A2:A10)</f>
         <v/>
       </c>
-      <c r="F2" s="5" t="n"/>
-      <c r="G2" s="5" t="n"/>
+      <c r="F2" s="4">
+        <f>MIN(B2:B10)</f>
+        <v/>
+      </c>
+      <c r="G2" s="4">
+        <f>MIN(C2:C10)</f>
+        <v/>
+      </c>
+      <c r="H2">
+        <f>AVERAGE(E2:G2)</f>
+        <v/>
+      </c>
     </row>
     <row r="3" ht="16.5" customHeight="1">
-      <c r="A3" s="5" t="n">
+      <c r="A3" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="B3" s="5" t="n">
+      <c r="B3" s="4" t="n">
         <v>93</v>
       </c>
-      <c r="C3" s="5" t="n">
+      <c r="C3" s="4" t="n">
         <v>77</v>
       </c>
     </row>
     <row r="4" ht="16.5" customHeight="1">
-      <c r="A4" s="5" t="n">
+      <c r="A4" s="4" t="n">
         <v>46</v>
       </c>
-      <c r="B4" s="5" t="n">
+      <c r="B4" s="4" t="n">
         <v>75</v>
       </c>
-      <c r="C4" s="5" t="n">
+      <c r="C4" s="4" t="n">
         <v>82</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="n">
+      <c r="A5" s="4" t="n">
         <v>54</v>
       </c>
-      <c r="B5" s="5" t="n">
+      <c r="B5" s="4" t="n">
         <v>87</v>
       </c>
-      <c r="C5" s="5" t="n">
+      <c r="C5" s="4" t="n">
         <v>22</v>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -610,13 +618,13 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="n">
+      <c r="A6" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="B6" s="5" t="n">
+      <c r="B6" s="4" t="n">
         <v>82</v>
       </c>
-      <c r="C6" s="5" t="n">
+      <c r="C6" s="4" t="n">
         <v>10</v>
       </c>
       <c r="E6" s="2" t="n">
@@ -630,46 +638,46 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="n">
+      <c r="A7" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="B7" s="5" t="n">
+      <c r="B7" s="4" t="n">
         <v>63</v>
       </c>
-      <c r="C7" s="5" t="n">
+      <c r="C7" s="4" t="n">
         <v>47</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="n">
+      <c r="A8" s="4" t="n">
         <v>74</v>
       </c>
-      <c r="B8" s="5" t="n">
+      <c r="B8" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="C8" s="5" t="n">
+      <c r="C8" s="4" t="n">
         <v>57</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="n">
+      <c r="A9" s="4" t="n">
         <v>94</v>
       </c>
-      <c r="B9" s="5" t="n">
+      <c r="B9" s="4" t="n">
         <v>26</v>
       </c>
-      <c r="C9" s="5" t="n">
+      <c r="C9" s="4" t="n">
         <v>14</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="n">
+      <c r="A10" s="4" t="n">
         <v>94</v>
       </c>
-      <c r="B10" s="5" t="n">
+      <c r="B10" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="C10" s="5" t="n">
+      <c r="C10" s="4" t="n">
         <v>61</v>
       </c>
     </row>
@@ -686,7 +694,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -699,7 +707,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -712,7 +720,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>